<commit_message>
Nowa realizacja Żoliborz, 10 zdjęć w hero, kancelaria usunięta
Karuzela hero: 15 slajdów (5 dotychczasowych + 10 nowych) wraz
z kropkami nawigacji.

Kancelaria prawna wypada całkowicie - podstrona, zdjęcia, kafelek
i odwołania w nawigacji. Jej miejsce zajmuje "Mieszkanie w Warszawie
(Żoliborz)" (120 m², 2019) z własną podstroną, galerią i materiałami.

Realizacje przenumerowane 01-04 w kolejności ze strony głównej,
nawigacja poprzednia/następna przebudowana pod nowy zestaw.
Nazwy i lokalizacje zaktualizowane z nowego arkusza.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dane-realizacji.xlsx
+++ b/dane-realizacji.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filip/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E964C79-3EA3-A047-87EE-C00D9D2FF29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F166609-8348-D140-8375-8FECCAF7DD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrukcja" sheetId="1" r:id="rId1"/>
     <sheet name="Mieszkanie w Olsztynie" sheetId="2" r:id="rId2"/>
-    <sheet name="Kancelaria prawna" sheetId="3" r:id="rId3"/>
+    <sheet name="mieszkanie pszasnyska" sheetId="3" r:id="rId3"/>
     <sheet name="Salon fryzjerski" sheetId="4" r:id="rId4"/>
     <sheet name="Mieszkanie" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -47,10 +47,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Miasto, np. Olsztyn. Bez adresu.</t>
         </r>
@@ -423,42 +422,224 @@
         <r>
           <rPr>
             <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Miasto, np. Olsztyn. Bez adresu.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sama liczba z jednostką, np. 68 m².</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rok zakończenia, np. 2025.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000005000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Co obejmowała realizacja. Oddzielaj przecinkami.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{24CF2890-25E5-1F43-A92B-7867AED39D78}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Krótkie zdanie pod tytułem na stronie.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000007000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Pełnymi zdaniami, bez list.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000008000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Pełnymi zdaniami. Akapit 2 może zostać pusty.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000009000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000A000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000B000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
             <color theme="1"/>
             <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Miasto, np. Olsztyn. Bez adresu.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Sama liczba z jednostką, np. 68 m².</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rok zakończenia, np. 2025.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000005000000}">
+          <t>HEX z krzyżykiem, np. #17181b.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{ADE307C3-2728-E648-B1BD-34E78E935775}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000D000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000E000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000F000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>HEX z krzyżykiem, np. #17181b.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000010000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Krótko, np. Faktura: lakier matowy grafitowy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000011000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000012000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000013000000}">
       <text>
         <r>
           <rPr>
@@ -468,11 +649,11 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Co obejmowała realizacja. Oddzielaj przecinkami.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000006000000}">
+          <t>HEX z krzyżykiem, np. #17181b.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000014000000}">
       <text>
         <r>
           <rPr>
@@ -482,257 +663,62 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Krótkie zdanie pod tytułem na stronie.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Pełnymi zdaniami, bez list.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000008000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Pełnymi zdaniami. Akapit 2 może zostać pusty.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000009000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+          <t>Krótko, np. Faktura: lakier matowy grafitowy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000015000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
         </r>
       </text>
     </comment>
-    <comment ref="C20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000A000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+    <comment ref="C23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000016000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000B000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000017000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>HEX z krzyżykiem, np. #17181b.</t>
         </r>
       </text>
     </comment>
-    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000C000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000018000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Krótko, np. Faktura: lakier matowy grafitowy.</t>
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000D000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000E000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000F000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>HEX z krzyżykiem, np. #17181b.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000010000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Krótko, np. Faktura: lakier matowy grafitowy.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000011000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000012000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000013000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>HEX z krzyżykiem, np. #17181b.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000014000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Krótko, np. Faktura: lakier matowy grafitowy.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000015000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Czego dotyczy, np. Fronty, Podłoga, Blat.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000016000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>Nazwa materiału, np. Lakier matowy grafitowy.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000017000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>HEX z krzyżykiem, np. #17181b.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000018000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Krótko, np. Faktura: lakier matowy grafitowy.</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="B28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000019000000}">
       <text>
         <r>
@@ -751,10 +737,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Co widać na zdjęciu. Czytają to niewidomi użytkownicy i Google.</t>
         </r>
@@ -765,10 +750,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Co widać na zdjęciu. Czytają to niewidomi użytkownicy i Google.</t>
         </r>
@@ -779,10 +763,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Co widać na zdjęciu. Czytają to niewidomi użytkownicy i Google.</t>
         </r>
@@ -803,10 +786,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Tytuł widoczny na stronie.</t>
         </r>
@@ -934,10 +916,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>HEX z krzyżykiem, np. #17181b.</t>
         </r>
@@ -1551,7 +1532,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="163">
   <si>
     <t>BAZZO INTERIORS — dane realizacji</t>
   </si>
@@ -1643,9 +1624,6 @@
     <t>Lokalizacja</t>
   </si>
   <si>
-    <t>Olsztyn</t>
-  </si>
-  <si>
     <t>Powierzchnia</t>
   </si>
   <si>
@@ -1700,39 +1678,21 @@
     <t>Opis zdjęcia faktury</t>
   </si>
   <si>
-    <t>Materiał 1</t>
-  </si>
-  <si>
     <t>#17181b</t>
   </si>
   <si>
-    <t>Materiał 2</t>
-  </si>
-  <si>
     <t>Podłoga</t>
   </si>
   <si>
     <t>#6d6964</t>
   </si>
   <si>
-    <t>Materiał 3</t>
-  </si>
-  <si>
     <t>#aca99e</t>
   </si>
   <si>
-    <t>Materiał 4</t>
-  </si>
-  <si>
-    <t>Marmur naturalny</t>
-  </si>
-  <si>
     <t>#8d867d</t>
   </si>
   <si>
-    <t>Faktura: marmur naturalny</t>
-  </si>
-  <si>
     <t>04 / GALERIA ZDJĘĆ  (do 4 pozycji)</t>
   </si>
   <si>
@@ -1742,99 +1702,36 @@
     <t>Opis zdjęcia (co widać na zdjęciu)</t>
   </si>
   <si>
-    <t>Zdjęcie 1</t>
-  </si>
-  <si>
-    <t>Zdjęcie 2</t>
-  </si>
-  <si>
-    <t>Zdjęcie 3</t>
-  </si>
-  <si>
     <t>Przedpokój z lustrzaną zabudową</t>
   </si>
   <si>
-    <t>Zdjęcie 4</t>
-  </si>
-  <si>
     <t>Zabudowa kuchenna z barem i hokerami</t>
   </si>
   <si>
     <t>REALIZACJA 02 — Kancelaria prawna</t>
   </si>
   <si>
-    <t>Kancelaria prawna</t>
-  </si>
-  <si>
-    <t>Projekt wnętrza, zabudowy stolarskie</t>
-  </si>
-  <si>
-    <t>Wnętrze biurowe z reprezentacyjną częścią dla klientów kancelarii.</t>
-  </si>
-  <si>
-    <t>Projekt łączy wymogi codziennej pracy z reprezentacyjnym charakterem miejsca, w którym przyjmowani są klienci. Ciemna ściana o wyrazistej fakturze wyznacza strefę spotkań i stanowi tło dla części wypoczynkowej.</t>
-  </si>
-  <si>
-    <t>Zabudowy stolarskie wykonano na wymiar, dopasowując je do proporcji pomieszczenia i porządkując przechowywanie dokumentów.</t>
-  </si>
-  <si>
     <t>Zdjęcia faktur → do-wrzucenia/kancelaria-prawna/materialy/  jako 1, 2, 3, 4</t>
   </si>
   <si>
-    <t>Okładzina</t>
-  </si>
-  <si>
-    <t>Kamień dekoracyjny łupany</t>
-  </si>
-  <si>
     <t>#46443f</t>
   </si>
   <si>
-    <t>Faktura: kamień dekoracyjny łupany</t>
-  </si>
-  <si>
-    <t>Deska warstwowa dębowa</t>
-  </si>
-  <si>
     <t>#c19665</t>
   </si>
   <si>
-    <t>Faktura: deska warstwowa dębowa</t>
-  </si>
-  <si>
-    <t>Tapicerka</t>
-  </si>
-  <si>
-    <t>Skóra naturalna pikowana</t>
-  </si>
-  <si>
     <t>#18181a</t>
   </si>
   <si>
-    <t>Faktura: skóra naturalna pikowana</t>
-  </si>
-  <si>
-    <t>Stolik</t>
-  </si>
-  <si>
     <t>#7a756c</t>
   </si>
   <si>
     <t>Zdjęcia → do-wrzucenia/kancelaria-prawna/galeria/  jako 1, 2, 3, 4.  Brak zdjęcia = zostaw wiersz pusty.</t>
   </si>
   <si>
-    <t>Strefa wypoczynkowa z ciemną sofą przy kamiennej ścianie</t>
-  </si>
-  <si>
-    <t>Część reprezentacyjna z granatową sofą i kamiennym stolikiem</t>
-  </si>
-  <si>
     <t>REALIZACJA 03 — Salon fryzjerski</t>
   </si>
   <si>
-    <t>Salon fryzjerski</t>
-  </si>
-  <si>
     <t>Projekt wnętrza, zabudowa stanowisk, kontuar</t>
   </si>
   <si>
@@ -1874,9 +1771,6 @@
     <t>REALIZACJA 04 — Mieszkanie</t>
   </si>
   <si>
-    <t>Mieszkanie</t>
-  </si>
-  <si>
     <t>Zdjęcia faktur → do-wrzucenia/mieszkanie/materialy/  jako 1, 2, 3, 4</t>
   </si>
   <si>
@@ -1910,9 +1804,6 @@
     <t>Zdjęcia → do-wrzucenia/mieszkanie/galeria/  jako 1, 2, 3, 4.  Brak zdjęcia = zostaw wiersz pusty.</t>
   </si>
   <si>
-    <t>Apartament w Olsztynie</t>
-  </si>
-  <si>
     <t>Projekt, meble na wymiar, zabduwowy stolarskie, wykończenie pod klucz</t>
   </si>
   <si>
@@ -1928,9 +1819,6 @@
     <t>Spiek kwarcowy</t>
   </si>
   <si>
-    <t>Faktura: Czarny spiek z białym użyleniem</t>
-  </si>
-  <si>
     <t>Strefa dzienna z panoramicznym przeszkleniem</t>
   </si>
   <si>
@@ -1940,24 +1828,15 @@
     <t>Zabudowa na korytarzu</t>
   </si>
   <si>
-    <t>Faktura: Jasna, dębowa podłoga w klasycznym układzie prostym.</t>
-  </si>
-  <si>
     <t>Hoker</t>
   </si>
   <si>
-    <t>Warszawa</t>
-  </si>
-  <si>
     <t>Wnętrze usługowe, w którym każdy element zabudowy musiał pogodzić wymagania techniczne z wyrazistym charakterem miejsca. Kontuar recepcji wykończono  patynowymi płytkami gresowymi, które nadają przestrzeni indywidualny rys.</t>
   </si>
   <si>
     <t>Patynowane płyty gresowe</t>
   </si>
   <si>
-    <t>Faktura: Patynowane płyty gresowe</t>
-  </si>
-  <si>
     <t>Zdjęcie 1 GPT</t>
   </si>
   <si>
@@ -1970,15 +1849,9 @@
     <t>Zdjęcie 6 GPT</t>
   </si>
   <si>
-    <t>Faktura: Lustrzana zabudowa na korytarzu</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alcantara </t>
   </si>
   <si>
-    <t xml:space="preserve">Faktura: Czarna alcantara </t>
-  </si>
-  <si>
     <t>Zabudowa ze stali nierdzewnej  na kosmetyki</t>
   </si>
   <si>
@@ -1991,25 +1864,16 @@
     <t>Stal nierdzewna</t>
   </si>
   <si>
-    <t>Zabudowa wykonana ze stali nierdzewnej</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ściana </t>
   </si>
   <si>
     <t xml:space="preserve">Blacha oksydowana </t>
   </si>
   <si>
-    <t>Blacha oksydowana, polakierowana na wysoki połysk</t>
-  </si>
-  <si>
     <t>Zabudowa na ubrania wierzchne</t>
   </si>
   <si>
     <t xml:space="preserve">Płyta MDF w czarnym macie </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Warszawa </t>
   </si>
   <si>
     <t>Realizacja skoncentrowana na strefie dziennej, gdzie meble, oświetlenie i wykończenia tworzą spójną, spokojną przestrzeń do codziennego życia.
@@ -2050,6 +1914,114 @@
   </si>
   <si>
     <t>Faktura: czarny spiek kwarcowy</t>
+  </si>
+  <si>
+    <t>Mieszkanie w Warszawie (Bielany)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warszawa - Bielany </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salon fryzjerski w Warszawie (Śródmieście)			</t>
+  </si>
+  <si>
+    <t>Warszawa - Śródmieście</t>
+  </si>
+  <si>
+    <t>Mieszkanie w Warszawie (Żoliborz)</t>
+  </si>
+  <si>
+    <t>Warszawa - Żoliborż</t>
+  </si>
+  <si>
+    <t>Mieszkanie w Olsztynie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projekt, meble na wymiar, zabduwowy stolarskie, wykończenie pod klucz			</t>
+  </si>
+  <si>
+    <t>Olsztyn - Śródmieście</t>
+  </si>
+  <si>
+    <t>Zdjęcie 69</t>
+  </si>
+  <si>
+    <t>Industrialna kuchnia z wyspą wykończoną mozaikowymi płytkami, surowym stalowym okapem i zabudową z betonowych płyt.</t>
+  </si>
+  <si>
+    <t>Zdjęcie 70</t>
+  </si>
+  <si>
+    <t>Zdjęcie 71</t>
+  </si>
+  <si>
+    <t>Stół z granitowym blatem na charakterystycznej, czarnej stalowej konstrukcji zestawiono z personalizowaną lampą chirurgiczną.</t>
+  </si>
+  <si>
+    <t>Zdjęcie 72</t>
+  </si>
+  <si>
+    <t>Przeszklone drzwi w czarnej, metalowej konstrukcji nadają wnętrzu nowoczesny, industrialny charakter.</t>
+  </si>
+  <si>
+    <t>Wnętrze mieszkalne, w którym surowe materiały zostały zestawione z prostą, funkcjonalną formą. Zabudowę wykonano z bejcowanej i lakierowanej płyty OSB, uzupełniając ją oksydowaną blachą, dekoracyjną mozaiką oraz czarnymi konstrukcjami metalowymi. Charakter wnętrza podkreślają również industrialne przeszklenia i indywidualnie zaprojektowane elementy wyposażenia. Zakres obejmował autorski projekt wnętrza, wykonanie mebli na wymiar oraz kompleksową realizację i koordynację prac wykończeniowych.</t>
+  </si>
+  <si>
+    <t>Zabudowa z bejcowanej i lakierowanej płyty OSB nadaje wnętrzu surowy, industrialny charakter, uzupełniony czarnymi detalami i dekoracyjną mozaiką. Całość dopełnia podłoga wykonana ze sklejki pokrytej filmem melaminowym.</t>
+  </si>
+  <si>
+    <t>Bejcowana i lakierowana płyta OSB</t>
+  </si>
+  <si>
+    <t>Płyty pokryte filmem melaminowym</t>
+  </si>
+  <si>
+    <t>Faktura: film melaminowy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zabudowa kuchenna </t>
+  </si>
+  <si>
+    <t>Betonowe płyty</t>
+  </si>
+  <si>
+    <t>Faktura: betonowe płyty</t>
+  </si>
+  <si>
+    <t>Faktura: bejcowana i lakierowana płyta OSB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faktura: czarna alcantara </t>
+  </si>
+  <si>
+    <t>Faktura: jasna, dębowa podłoga w klasycznym układzie prostym.</t>
+  </si>
+  <si>
+    <t>Faktura: patynowane płyty gresowe</t>
+  </si>
+  <si>
+    <t>Faktura: zabudowa wykonana ze stali nierdzewnej</t>
+  </si>
+  <si>
+    <t>Faktura: blacha oksydowana, polakierowana na wysoki połysk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faktura: płyta MDF w czarnym macie </t>
+  </si>
+  <si>
+    <t>Faktura: czarny spiek z białym użyleniem</t>
+  </si>
+  <si>
+    <t>Faktura: lustrzana zabudowa na korytarzu</t>
+  </si>
+  <si>
+    <t>Stół</t>
+  </si>
+  <si>
+    <t>Ciemny granit</t>
+  </si>
+  <si>
+    <t>Faktura: Ciemny granit</t>
   </si>
 </sst>
 </file>
@@ -2260,18 +2232,18 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2720,13 +2692,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -2748,79 +2720,79 @@
       <c r="A5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
+      <c r="B5" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="B6" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="18">
+        <v>30</v>
+      </c>
+      <c r="B7" s="12">
         <v>140</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="18">
+        <v>31</v>
+      </c>
+      <c r="B8" s="12">
         <v>2025</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="16"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
+        <v>32</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -2828,55 +2800,55 @@
     </row>
     <row r="14" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+        <v>40</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="16" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>47</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2884,16 +2856,16 @@
         <v>2</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2901,16 +2873,16 @@
         <v>4</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2918,16 +2890,16 @@
         <v>7</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2935,38 +2907,38 @@
         <v>9</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
@@ -2974,50 +2946,57 @@
     </row>
     <row r="28" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="16"/>
+        <v>101</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="16"/>
+        <v>102</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="16"/>
+        <v>103</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="16"/>
+        <v>104</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B8:E8"/>
@@ -3026,13 +3005,6 @@
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Nieprawidłowy kod koloru" error="Kod musi mieć format #rrggbb — krzyżyk i 6 znaków, np. #17181b." sqref="D20:D23" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -3040,6 +3012,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -3057,13 +3030,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="A1" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -3085,73 +3058,79 @@
       <c r="A5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
+      <c r="B5" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="B6" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+        <v>30</v>
+      </c>
+      <c r="B7" s="12">
+        <v>120</v>
+      </c>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="16"/>
+        <v>31</v>
+      </c>
+      <c r="B8" s="12">
+        <v>2019</v>
+      </c>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
+        <v>32</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -3159,145 +3138,143 @@
     </row>
     <row r="14" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
+        <v>38</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+        <v>40</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
+      <c r="A18" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>48</v>
-      </c>
     </row>
     <row r="20" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="10">
+        <v>55</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="10">
+        <v>56</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>52</v>
-      </c>
       <c r="C21" s="9" t="s">
-        <v>80</v>
+        <v>146</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>82</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10" t="s">
-        <v>54</v>
+      <c r="A22" s="10">
+        <v>57</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>83</v>
+        <v>148</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>84</v>
+        <v>149</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
-        <v>56</v>
+      <c r="A23" s="10">
+        <v>58</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>87</v>
+        <v>160</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>57</v>
+        <v>161</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>59</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
@@ -3305,46 +3282,57 @@
     </row>
     <row r="28" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="16"/>
+        <v>136</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="16"/>
+        <v>138</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="16"/>
+        <v>139</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="16"/>
+        <v>141</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B8:E8"/>
@@ -3353,13 +3341,6 @@
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Nieprawidłowy kod koloru" error="Kod musi mieć format #rrggbb — krzyżyk i 6 znaków, np. #17181b." sqref="D20:D23" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -3384,13 +3365,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="A1" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -3412,79 +3393,79 @@
       <c r="A5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
+      <c r="B5" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="B6" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="18">
+        <v>30</v>
+      </c>
+      <c r="B7" s="12">
         <v>200</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="18">
+        <v>31</v>
+      </c>
+      <c r="B8" s="12">
         <v>2022</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="16"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
+        <v>32</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
+        <v>33</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -3492,55 +3473,55 @@
     </row>
     <row r="14" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
+        <v>38</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+        <v>40</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
+      <c r="A18" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>47</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3548,16 +3529,16 @@
         <v>11</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>133</v>
+        <v>100</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>99</v>
+        <v>71</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3565,16 +3546,16 @@
         <v>12</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3582,16 +3563,16 @@
         <v>13</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>147</v>
+        <v>110</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>148</v>
+        <v>111</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3599,38 +3580,38 @@
         <v>14</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>151</v>
+        <v>113</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>103</v>
+        <v>75</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
@@ -3640,48 +3621,55 @@
       <c r="A28" s="10">
         <v>30</v>
       </c>
-      <c r="B28" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="16"/>
+      <c r="B28" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
         <v>31</v>
       </c>
-      <c r="B29" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="16"/>
+      <c r="B29" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
         <v>32</v>
       </c>
-      <c r="B30" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="16"/>
+      <c r="B30" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
         <v>33</v>
       </c>
-      <c r="B31" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="16"/>
+      <c r="B31" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B8:E8"/>
@@ -3690,13 +3678,6 @@
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Nieprawidłowy kod koloru" error="Kod musi mieć format #rrggbb — krzyżyk i 6 znaków, np. #17181b." sqref="D20:D23" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -3721,13 +3702,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="A1" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -3749,79 +3730,79 @@
       <c r="A5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
+      <c r="B5" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="B6" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="18">
+        <v>30</v>
+      </c>
+      <c r="B7" s="12">
         <v>70</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="18">
+        <v>31</v>
+      </c>
+      <c r="B8" s="12">
         <v>2024</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="16"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
+        <v>32</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -3829,55 +3810,55 @@
     </row>
     <row r="14" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
+        <v>38</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+        <v>40</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
+      <c r="A18" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>47</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3885,16 +3866,16 @@
         <v>111</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>163</v>
+        <v>124</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>164</v>
+        <v>125</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3902,16 +3883,16 @@
         <v>112</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>110</v>
+        <v>81</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3919,16 +3900,16 @@
         <v>113</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>165</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3936,38 +3917,38 @@
         <v>114</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
@@ -3975,50 +3956,57 @@
     </row>
     <row r="28" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="16"/>
+        <v>119</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="16"/>
+        <v>116</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="16"/>
+        <v>120</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B31" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="16"/>
+        <v>122</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B8:E8"/>
@@ -4027,13 +4015,6 @@
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Nieprawidłowy kod koloru" error="Kod musi mieć format #rrggbb — krzyżyk i 6 znaków, np. #17181b." sqref="D20:D23" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>